<commit_message>
S78: stage two client emails for Bill - the 224-row workbook and the lead-count correction
</commit_message>
<xml_diff>
--- a/mail/NCC-HOA-Directory-Workbook.xlsx
+++ b/mail/NCC-HOA-Directory-Workbook.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Dev-lead cross-ref" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All associations'!$A$1:$N$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All associations'!$A$1:$N$225</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tier 1 - call these first'!$A$1:$N$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -526,7 +526,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Tier 2 — self-managed, no email on file           99   ← reachable by mail or phone; email still to find</t>
+          <t xml:space="preserve">  Tier 2 — self-managed, no email on file          100   ← reachable by mail or phone; email still to find</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Total in this workbook                           223</t>
+          <t xml:space="preserve">  Total in this workbook                           224</t>
         </is>
       </c>
     </row>
@@ -557,49 +557,45 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1. The county directory publishes 224 associations. This workbook has 223.</t>
+          <t>1. This is the complete directory: all 224 associations the county publishes are</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">   One directory row is a New Castle association called Hunters Ridge. A community of the</t>
+          <t xml:space="preserve">   in this workbook, none omitted.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   same name exists in Kent County and is already one of your warm leads. The two were</t>
-        </is>
-      </c>
+      <c r="A18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   briefly merged in our records on 25 Aug and were separated again the same day, so the</t>
+          <t xml:space="preserve">   One name to watch — there are two communities called Hunters Ridge in Delaware, one</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Kent record now carries its own president again. The New Castle Hunters Ridge does not</t>
+          <t xml:space="preserve">   here in New Castle County and one in Kent that is already a warm lead of yours. They</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   yet have its own record here — it is the one row missing, and it is a known gap, not a</t>
+          <t xml:space="preserve">   are different associations with different boards, and we keep them as separate records.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">   silent one.</t>
+          <t xml:space="preserve">   The Hunters Ridge in this workbook is the New Castle one.</t>
         </is>
       </c>
     </row>
@@ -697,7 +693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N224"/>
+  <dimension ref="A1:N225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6895,7 +6891,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Kendall</t>
+          <t>Hunters Ridge</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -6905,12 +6901,12 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Jeff Miller, President</t>
+          <t>Daniel Kennefick, President</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>4 Kendall Court, Wilmington, DE 19803</t>
+          <t>P.O. Box 15020, Newark, DE 19711</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
@@ -6932,7 +6928,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Kensington</t>
+          <t>Kendall</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -6942,17 +6938,12 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Katherine Ennis, President</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>302-563-2305</t>
+          <t>Jeff Miller, President</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
         <is>
-          <t>25 Lochview Drive, Bear, DE 19701</t>
+          <t>4 Kendall Court, Wilmington, DE 19803</t>
         </is>
       </c>
       <c r="M135" t="inlineStr">
@@ -6974,7 +6965,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Kentmere</t>
+          <t>Kensington</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -6984,12 +6975,17 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Judy Sharp, President</t>
+          <t>Katherine Ennis, President</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>302-563-2305</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>828 Old Harmony Road, Newark, DE 19711</t>
+          <t>25 Lochview Drive, Bear, DE 19701</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
@@ -7011,7 +7007,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Lea Eara Farms</t>
+          <t>Kentmere</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -7021,32 +7017,22 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Charles Layton, President</t>
-        </is>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>MIDDLETOWN</t>
-        </is>
-      </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>19709</t>
-        </is>
-      </c>
-      <c r="L137" t="inlineStr">
-        <is>
-          <t>154</t>
+          <t>Judy Sharp, President</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>828 Old Harmony Road, Newark, DE 19711</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N137" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -7058,7 +7044,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Lums Pond Estates III</t>
+          <t>Lea Eara Farms</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -7068,22 +7054,32 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Tom Thomas, President</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr">
-        <is>
-          <t>408 Cheer Court, Bear, DE 19701</t>
+          <t>Charles Layton, President</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>MIDDLETOWN</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>19709</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>154</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N138" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -7095,7 +7091,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Lums Pond Estates IV</t>
+          <t>Lums Pond Estates III</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -7105,12 +7101,12 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Vincent Johnson, President</t>
+          <t>Tom Thomas, President</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>206 Olivia Way, Bear, DE 19701</t>
+          <t>408 Cheer Court, Bear, DE 19701</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -7132,7 +7128,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Mariners Watch</t>
+          <t>Lums Pond Estates IV</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -7142,12 +7138,12 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Michael Jones, President</t>
+          <t>Vincent Johnson, President</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>P.O. Box 387, Bear, DE 19701</t>
+          <t>206 Olivia Way, Bear, DE 19701</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
@@ -7169,7 +7165,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Meadowdale</t>
+          <t>Mariners Watch</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -7179,12 +7175,12 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Ian Heringslack, President</t>
+          <t>Michael Jones, President</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>21 Donegal Court, Newark, DE 19711</t>
+          <t>P.O. Box 387, Bear, DE 19701</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -7206,7 +7202,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Merestone</t>
+          <t>Meadowdale</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -7216,12 +7212,12 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Alexander Selimov, President</t>
+          <t>Ian Heringslack, President</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>5 Reese Drive, Newark, DE 19711</t>
+          <t>21 Donegal Court, Newark, DE 19711</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
@@ -7243,7 +7239,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Midvale Addition</t>
+          <t>Merestone</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -7253,12 +7249,12 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Juantia Fletcher, Treasurer</t>
+          <t>Alexander Selimov, President</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>105 6th Avenue, New Castle, DE 19720</t>
+          <t>5 Reese Drive, Newark, DE 19711</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
@@ -7280,7 +7276,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Millwood</t>
+          <t>Midvale Addition</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -7290,12 +7286,12 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Edward Schwar, President</t>
+          <t>Juantia Fletcher, Treasurer</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>52 Millwood Drive, Middletown, DE 19709</t>
+          <t>105 6th Avenue, New Castle, DE 19720</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
@@ -7317,7 +7313,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Nonantum Mills</t>
+          <t>Millwood</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -7327,12 +7323,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Timothy Reighart, President</t>
+          <t>Edward Schwar, President</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>P.O. Box 9652, Newark, DE 19714</t>
+          <t>52 Millwood Drive, Middletown, DE 19709</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
@@ -7354,7 +7350,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Nordic Dell</t>
+          <t>Nonantum Mills</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -7364,12 +7360,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>David Donohue, President</t>
+          <t>Timothy Reighart, President</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>106 Carriage Way, Wilmington, DE 19803</t>
+          <t>P.O. Box 9652, Newark, DE 19714</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -7391,7 +7387,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Penn Manor</t>
+          <t>Nordic Dell</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -7401,12 +7397,12 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Evan Kenney, President</t>
+          <t>David Donohue, President</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>450 Coldspring Run, Newark, DE 19711</t>
+          <t>106 Carriage Way, Wilmington, DE 19803</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -7428,7 +7424,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Pierson Farm</t>
+          <t>Penn Manor</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -7438,32 +7434,22 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Jeffrey Goldstein, President</t>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr">
-        <is>
-          <t>WILMINGTON</t>
-        </is>
-      </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>19810</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>70</t>
+          <t>Evan Kenney, President</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>450 Coldspring Run, Newark, DE 19711</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N148" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -7475,7 +7461,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Piersons Ridge</t>
+          <t>Pierson Farm</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -7485,22 +7471,22 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Jingkun Li, Vice President</t>
+          <t>Jeffrey Goldstein, President</t>
         </is>
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>HOCKESSIN</t>
+          <t>WILMINGTON</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
         <is>
-          <t>19707</t>
+          <t>19810</t>
         </is>
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>70</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
@@ -7522,7 +7508,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Pine Tree Estates</t>
+          <t>Piersons Ridge</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -7532,22 +7518,22 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Peggy Gladstone, Treasurer</t>
+          <t>Jingkun Li, Vice President</t>
         </is>
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>TOWNSEND</t>
+          <t>HOCKESSIN</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>19734</t>
+          <t>19707</t>
         </is>
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>98</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
@@ -7569,7 +7555,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Preserve at Presidential Estates</t>
+          <t>Pine Tree Estates</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -7579,22 +7565,32 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Jeffrey Karron, President</t>
-        </is>
-      </c>
-      <c r="H151" t="inlineStr">
-        <is>
-          <t>21 Emsley Drive, Wilmington, DE 19810</t>
+          <t>Peggy Gladstone, Treasurer</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>TOWNSEND</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>19734</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>21</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N151" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -7606,7 +7602,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Radnor Green</t>
+          <t>Preserve at Presidential Estates</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -7616,37 +7612,22 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Beth Bonsall, President</t>
-        </is>
-      </c>
-      <c r="I152" t="inlineStr">
-        <is>
-          <t>https://radnorgreencivic.com</t>
-        </is>
-      </c>
-      <c r="J152" t="inlineStr">
-        <is>
-          <t>CLAYMONT</t>
-        </is>
-      </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>19703</t>
-        </is>
-      </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>176</t>
+          <t>Jeffrey Karron, President</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>21 Emsley Drive, Wilmington, DE 19810</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N152" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7639,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Ramsey Ridge</t>
+          <t>Radnor Green</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -7668,22 +7649,27 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Jason Williams, President</t>
+          <t>Beth Bonsall, President</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>https://radnorgreencivic.com</t>
         </is>
       </c>
       <c r="J153" t="inlineStr">
         <is>
-          <t>HOCKESSIN</t>
+          <t>CLAYMONT</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>19707</t>
+          <t>19703</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>176</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
@@ -7705,7 +7691,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Reserve at Hockessin Chase</t>
+          <t>Ramsey Ridge</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -7715,22 +7701,32 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Baqar Shameem, President</t>
-        </is>
-      </c>
-      <c r="H154" t="inlineStr">
-        <is>
-          <t>32 Harvest Lane, Hockessin, DE 19707</t>
+          <t>Jason Williams, President</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>HOCKESSIN</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>19707</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>91</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N154" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -7742,7 +7738,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Reserve At Ironside</t>
+          <t>Reserve at Hockessin Chase</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -7752,32 +7748,22 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Rick Lightle, President</t>
-        </is>
-      </c>
-      <c r="J155" t="inlineStr">
-        <is>
-          <t>NEWARK</t>
-        </is>
-      </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>19702</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>87</t>
+          <t>Baqar Shameem, President</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>32 Harvest Lane, Hockessin, DE 19707</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -7789,7 +7775,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Richards Lane</t>
+          <t>Reserve At Ironside</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -7799,22 +7785,32 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Carolyn Dehorty, President</t>
-        </is>
-      </c>
-      <c r="H156" t="inlineStr">
-        <is>
-          <t>123 Richards Lane, Newark, DE 19711</t>
+          <t>Rick Lightle, President</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>NEWARK</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>19702</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>87</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -7826,7 +7822,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Sanford Ridge</t>
+          <t>Richards Lane</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -7836,32 +7832,22 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Larry Rufo, President</t>
-        </is>
-      </c>
-      <c r="J157" t="inlineStr">
-        <is>
-          <t>HOCKESSIN</t>
-        </is>
-      </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>19707</t>
-        </is>
-      </c>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>74</t>
+          <t>Carolyn Dehorty, President</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>123 Richards Lane, Newark, DE 19711</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N157" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -7873,7 +7859,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Sharpley</t>
+          <t>Sanford Ridge</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -7883,22 +7869,32 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Marilyn McGowan, President</t>
-        </is>
-      </c>
-      <c r="H158" t="inlineStr">
-        <is>
-          <t>617 Haverhill Road, Wilmington, DE 19803</t>
+          <t>Larry Rufo, President</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>HOCKESSIN</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>19707</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>74</t>
         </is>
       </c>
       <c r="M158" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N158" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -7910,7 +7906,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Shipley Chase</t>
+          <t>Sharpley</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -7920,32 +7916,22 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Marylou Sinko, President</t>
-        </is>
-      </c>
-      <c r="J159" t="inlineStr">
-        <is>
-          <t>WILMINGTON</t>
-        </is>
-      </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>19810</t>
-        </is>
-      </c>
-      <c r="L159" t="inlineStr">
-        <is>
-          <t>9</t>
+          <t>Marilyn McGowan, President</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>617 Haverhill Road, Wilmington, DE 19803</t>
         </is>
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N159" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -7957,7 +7943,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Southbridge</t>
+          <t>Shipley Chase</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7967,22 +7953,32 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Maria Reed, President</t>
-        </is>
-      </c>
-      <c r="H160" t="inlineStr">
-        <is>
-          <t>1218 B Street, Wilmington, DE 19802</t>
+          <t>Marylou Sinko, President</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>WILMINGTON</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>19810</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N160" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -7994,7 +7990,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Southwood Estates</t>
+          <t>Southbridge</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -8004,32 +8000,22 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Michael Terranova, President</t>
-        </is>
-      </c>
-      <c r="J161" t="inlineStr">
-        <is>
-          <t>HOCKESSIN</t>
-        </is>
-      </c>
-      <c r="K161" t="inlineStr">
-        <is>
-          <t>19707</t>
-        </is>
-      </c>
-      <c r="L161" t="inlineStr">
-        <is>
-          <t>61</t>
+          <t>Maria Reed, President</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>1218 B Street, Wilmington, DE 19802</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8041,7 +8027,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Springer Woods</t>
+          <t>Southwood Estates</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -8051,22 +8037,32 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Don Schuler, President</t>
-        </is>
-      </c>
-      <c r="H162" t="inlineStr">
-        <is>
-          <t>236 Hoyer Court, Wilmington, DE 19803</t>
+          <t>Michael Terranova, President</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>HOCKESSIN</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>19707</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>61</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8074,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Stonefield</t>
+          <t>Springer Woods</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -8088,12 +8084,12 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Richard Wagner, President</t>
+          <t>Don Schuler, President</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>P.O. Box 316, Middletown, DE 19709</t>
+          <t>236 Hoyer Court, Wilmington, DE 19803</t>
         </is>
       </c>
       <c r="M163" t="inlineStr">
@@ -8115,7 +8111,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Summit Pond</t>
+          <t>Stonefield</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -8125,32 +8121,22 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>William Krespan Jr., President</t>
-        </is>
-      </c>
-      <c r="J164" t="inlineStr">
-        <is>
-          <t>MIDDLETOWN</t>
-        </is>
-      </c>
-      <c r="K164" t="inlineStr">
-        <is>
-          <t>19709</t>
-        </is>
-      </c>
-      <c r="L164" t="inlineStr">
-        <is>
-          <t>60</t>
+          <t>Richard Wagner, President</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>P.O. Box 316, Middletown, DE 19709</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N164" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8162,7 +8148,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Sunrise Court</t>
+          <t>Summit Pond</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -8172,22 +8158,22 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>James Gates, President</t>
+          <t>William Krespan Jr., President</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
         <is>
-          <t>NEWARK</t>
+          <t>MIDDLETOWN</t>
         </is>
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>19713</t>
+          <t>19709</t>
         </is>
       </c>
       <c r="L165" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>60</t>
         </is>
       </c>
       <c r="M165" t="inlineStr">
@@ -8209,7 +8195,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Tall Pines</t>
+          <t>Sunrise Court</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -8219,22 +8205,32 @@
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>Jeffrey Biddle, President</t>
-        </is>
-      </c>
-      <c r="H166" t="inlineStr">
-        <is>
-          <t>148 Tall Pines Road, Newark, DE 19713</t>
+          <t>James Gates, President</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>NEWARK</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>19713</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N166" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8242,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Tall Trees</t>
+          <t>Tall Pines</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -8256,12 +8252,12 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>Donald Nayden, President</t>
+          <t>Jeffrey Biddle, President</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>11 Tall Trees Lane, Wilmington, DE 19808</t>
+          <t>148 Tall Pines Road, Newark, DE 19713</t>
         </is>
       </c>
       <c r="M167" t="inlineStr">
@@ -8283,7 +8279,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>The Oaks</t>
+          <t>Tall Trees</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -8293,12 +8289,12 @@
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>Richard Houtz, President</t>
+          <t>Donald Nayden, President</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>2 Split Rail Lane, Newark, DE 19702</t>
+          <t>11 Tall Trees Lane, Wilmington, DE 19808</t>
         </is>
       </c>
       <c r="M168" t="inlineStr">
@@ -8320,7 +8316,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Thomas Pointe</t>
+          <t>The Oaks</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -8330,32 +8326,22 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Tammy Quig, Treasurer</t>
-        </is>
-      </c>
-      <c r="J169" t="inlineStr">
-        <is>
-          <t>WILMINGTON</t>
-        </is>
-      </c>
-      <c r="K169" t="inlineStr">
-        <is>
-          <t>19808</t>
-        </is>
-      </c>
-      <c r="L169" t="inlineStr">
-        <is>
-          <t>20</t>
+          <t>Richard Houtz, President</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>2 Split Rail Lane, Newark, DE 19702</t>
         </is>
       </c>
       <c r="M169" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8367,7 +8353,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Timber Farms</t>
+          <t>Thomas Pointe</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -8377,22 +8363,22 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Rolf Joerger, President</t>
+          <t>Tammy Quig, Treasurer</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>NEWARK</t>
+          <t>WILMINGTON</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>19702</t>
+          <t>19808</t>
         </is>
       </c>
       <c r="L170" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>20</t>
         </is>
       </c>
       <c r="M170" t="inlineStr">
@@ -8414,7 +8400,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Traditions At Jester Crossing</t>
+          <t>Timber Farms</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -8424,22 +8410,22 @@
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>Helen Monroe, President</t>
+          <t>Rolf Joerger, President</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
         <is>
-          <t>BEAR</t>
+          <t>NEWARK</t>
         </is>
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>19701</t>
+          <t>19702</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>71</t>
         </is>
       </c>
       <c r="M171" t="inlineStr">
@@ -8461,7 +8447,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Village Of Red Lion Creek</t>
+          <t>Traditions At Jester Crossing</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -8471,7 +8457,7 @@
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>Patricia Jones, President</t>
+          <t>Helen Monroe, President</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -8486,7 +8472,7 @@
       </c>
       <c r="L172" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>58</t>
         </is>
       </c>
       <c r="M172" t="inlineStr">
@@ -8508,7 +8494,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Welsh Hill Preserve</t>
+          <t>Village Of Red Lion Creek</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -8518,22 +8504,32 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Michael Brooks, President</t>
-        </is>
-      </c>
-      <c r="H173" t="inlineStr">
-        <is>
-          <t>P.O. Box 7644, Newark, DE 19714-7644</t>
+          <t>Patricia Jones, President</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>BEAR</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>19701</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>89</t>
         </is>
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N173" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -8545,7 +8541,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Westover Hills Section A</t>
+          <t>Welsh Hill Preserve</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -8555,12 +8551,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Eric Holloway, President</t>
+          <t>Michael Brooks, President</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>705 Edgehill Road, Wilmington, DE 19807</t>
+          <t>P.O. Box 7644, Newark, DE 19714-7644</t>
         </is>
       </c>
       <c r="M174" t="inlineStr">
@@ -8582,7 +8578,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Wood Creek</t>
+          <t>Westover Hills Section A</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -8592,17 +8588,12 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Ryan Coyne, Vice President</t>
+          <t>Eric Holloway, President</t>
         </is>
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>P.O. Box 142, Hockessin, DE 19707</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr">
-        <is>
-          <t>https://woodcreekcivic.org</t>
+          <t>705 Edgehill Road, Wilmington, DE 19807</t>
         </is>
       </c>
       <c r="M175" t="inlineStr">
@@ -8624,7 +8615,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Woods At Limestone Hills</t>
+          <t>Wood Creek</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -8634,17 +8625,27 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Kevin Walker, President</t>
+          <t>Ryan Coyne, Vice President</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>P.O. Box 142, Hockessin, DE 19707</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>https://woodcreekcivic.org</t>
         </is>
       </c>
       <c r="M176" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N176" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8656,7 +8657,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Wynnwood</t>
+          <t>Woods At Limestone Hills</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -8666,22 +8667,17 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Jimmy Marini, President</t>
-        </is>
-      </c>
-      <c r="H177" t="inlineStr">
-        <is>
-          <t>2312 Kennwynn Road, Wilmington, DE 19810</t>
+          <t>Kevin Walker, President</t>
         </is>
       </c>
       <c r="M177" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N177" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -8693,7 +8689,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Yardley Place</t>
+          <t>Wynnwood</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -8703,32 +8699,22 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Patrick Brunner, President</t>
-        </is>
-      </c>
-      <c r="J178" t="inlineStr">
-        <is>
-          <t>WILMINGTON</t>
-        </is>
-      </c>
-      <c r="K178" t="inlineStr">
-        <is>
-          <t>19810</t>
-        </is>
-      </c>
-      <c r="L178" t="inlineStr">
-        <is>
-          <t>25</t>
+          <t>Jimmy Marini, President</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>2312 Kennwynn Road, Wilmington, DE 19810</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N178" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8740,94 +8726,89 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
+          <t>Yardley Place</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>self-managed (no management company listed) [named officer listed]</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Patrick Brunner, President</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>WILMINGTON</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>19810</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>nccde_parcel_subdiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>2 - self-managed, no email</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
           <t>York Farms</t>
         </is>
       </c>
-      <c r="C179" t="inlineStr">
-        <is>
-          <t>self-managed (no management company listed) [named officer listed]</t>
-        </is>
-      </c>
-      <c r="E179" t="inlineStr">
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>self-managed (no management company listed) [named officer listed]</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
         <is>
           <t>Sidney Lewinson, President</t>
         </is>
       </c>
-      <c r="J179" t="inlineStr">
+      <c r="J180" t="inlineStr">
         <is>
           <t>BEAR</t>
         </is>
       </c>
-      <c r="K179" t="inlineStr">
+      <c r="K180" t="inlineStr">
         <is>
           <t>19701</t>
         </is>
       </c>
-      <c r="L179" t="inlineStr">
+      <c r="L180" t="inlineStr">
         <is>
           <t>115</t>
         </is>
       </c>
-      <c r="M179" t="inlineStr">
+      <c r="M180" t="inlineStr">
         <is>
           <t>cold</t>
         </is>
       </c>
-      <c r="N179" t="inlineStr">
+      <c r="N180" t="inlineStr">
         <is>
           <t>nccde_parcel_subdiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="5" t="inlineStr">
-        <is>
-          <t>3 - professionally managed</t>
-        </is>
-      </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>Academy Hills Phase V</t>
-        </is>
-      </c>
-      <c r="C180" t="inlineStr">
-        <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
-        </is>
-      </c>
-      <c r="D180" t="inlineStr">
-        <is>
-          <t>Aspen Property Management, MC</t>
-        </is>
-      </c>
-      <c r="F180" t="inlineStr">
-        <is>
-          <t>info@aspenpropertymgmt.com</t>
-        </is>
-      </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>410-620-2598</t>
-        </is>
-      </c>
-      <c r="H180" t="inlineStr">
-        <is>
-          <t>14 S Main Street, North East, MD 21901</t>
-        </is>
-      </c>
-      <c r="I180" t="inlineStr">
-        <is>
-          <t>https://www.aspenpropertymgmt.com</t>
-        </is>
-      </c>
-      <c r="M180" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="N180" t="inlineStr">
-        <is>
-          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8839,32 +8820,47 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Adams Run</t>
+          <t>Academy Hills Phase V</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>professionally managed (Mastriana Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Mastriana Property Management, MC</t>
+          <t>Aspen Property Management, MC</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>302-234-4860</t>
+          <t>410-620-2598</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>14 S Main Street, North East, MD 21901</t>
+        </is>
+      </c>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="M181" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N181" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -8876,7 +8872,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Adare Village</t>
+          <t>Adams Run</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -8892,21 +8888,6 @@
       <c r="G182" t="inlineStr">
         <is>
           <t>302-234-4860</t>
-        </is>
-      </c>
-      <c r="J182" t="inlineStr">
-        <is>
-          <t>HOCKESSIN</t>
-        </is>
-      </c>
-      <c r="K182" t="inlineStr">
-        <is>
-          <t>19707</t>
-        </is>
-      </c>
-      <c r="L182" t="inlineStr">
-        <is>
-          <t>53</t>
         </is>
       </c>
       <c r="M182" t="inlineStr">
@@ -8928,52 +8909,47 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Antrim</t>
+          <t>Adare Village</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
+          <t>professionally managed (Mastriana Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="E183" t="inlineStr">
-        <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="F183" t="inlineStr">
-        <is>
-          <t>steve@neighborhoodresources.net</t>
+          <t>Mastriana Property Management, MC</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>302-521-1961</t>
-        </is>
-      </c>
-      <c r="H183" t="inlineStr">
-        <is>
-          <t>P.O. Box 10012, Wilmington, DE 19850</t>
-        </is>
-      </c>
-      <c r="I183" t="inlineStr">
-        <is>
-          <t>https://neighborhoodresources.net</t>
+          <t>302-234-4860</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr">
+        <is>
+          <t>HOCKESSIN</t>
+        </is>
+      </c>
+      <c r="K183" t="inlineStr">
+        <is>
+          <t>19707</t>
+        </is>
+      </c>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>53</t>
         </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N183" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -8985,7 +8961,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Augustine Creek</t>
+          <t>Antrim</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -9013,34 +8989,24 @@
           <t>302-521-1961</t>
         </is>
       </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>P.O. Box 10012, Wilmington, DE 19850</t>
+        </is>
+      </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>http://www.augustinecreekde.com/</t>
-        </is>
-      </c>
-      <c r="J184" t="inlineStr">
-        <is>
-          <t>MIDDLETOWN</t>
-        </is>
-      </c>
-      <c r="K184" t="inlineStr">
-        <is>
-          <t>19709</t>
-        </is>
-      </c>
-      <c r="L184" t="inlineStr">
-        <is>
-          <t>32</t>
+          <t>https://neighborhoodresources.net</t>
         </is>
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -9052,7 +9018,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Augustine Creek II</t>
+          <t>Augustine Creek</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -9097,7 +9063,7 @@
       </c>
       <c r="L185" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>32</t>
         </is>
       </c>
       <c r="M185" t="inlineStr">
@@ -9119,47 +9085,62 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Ballymeade</t>
+          <t>Augustine Creek II</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>professionally managed (Penco Management Inc., MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
         </is>
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Penco Management Inc., MC</t>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>rwhite@pencomanagement.co</t>
+          <t>steve@neighborhoodresources.net</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>610-358-5580</t>
-        </is>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>5 Christy Drive, Chadds Ford, PA 19317</t>
+          <t>302-521-1961</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>https://www.ballymeade.org</t>
+          <t>http://www.augustinecreekde.com/</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr">
+        <is>
+          <t>MIDDLETOWN</t>
+        </is>
+      </c>
+      <c r="K186" t="inlineStr">
+        <is>
+          <t>19709</t>
+        </is>
+      </c>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>189</t>
         </is>
       </c>
       <c r="M186" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -9171,57 +9152,47 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Barbs Farm</t>
+          <t>Ballymeade</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Penco Management Inc., MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Penco Management Inc., MC</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>rwhite@pencomanagement.co</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
+          <t>610-358-5580</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>5 Christy Drive, Chadds Ford, PA 19317</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>https://www.aspenpropertymgmt.com</t>
-        </is>
-      </c>
-      <c r="J187" t="inlineStr">
-        <is>
-          <t>NEW CASTLE</t>
-        </is>
-      </c>
-      <c r="K187" t="inlineStr">
-        <is>
-          <t>19720</t>
-        </is>
-      </c>
-      <c r="L187" t="inlineStr">
-        <is>
-          <t>89</t>
+          <t>https://www.ballymeade.org</t>
         </is>
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N187" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -9233,27 +9204,32 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Bear Crossing</t>
+          <t>Barbs Farm</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>professionally managed (Investment Property Services, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Investment Property Services, MC</t>
+          <t>Aspen Property Management, MC</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>cperonti@ipsde.com</t>
+          <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>302-994-3907</t>
+          <t>410-620-2598</t>
+        </is>
+      </c>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -9268,7 +9244,7 @@
       </c>
       <c r="L188" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>89</t>
         </is>
       </c>
       <c r="M188" t="inlineStr">
@@ -9290,47 +9266,42 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Brennan Estates</t>
+          <t>Bear Crossing</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Investment Property Services, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Investment Property Services, MC</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>cperonti@ipsde.com</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr">
-        <is>
-          <t>https://brennanestatesassociation.org</t>
+          <t>302-994-3907</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
         <is>
-          <t>BEAR</t>
+          <t>NEW CASTLE</t>
         </is>
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>19701</t>
+          <t>19720</t>
         </is>
       </c>
       <c r="L189" t="inlineStr">
         <is>
-          <t>831</t>
+          <t>60</t>
         </is>
       </c>
       <c r="M189" t="inlineStr">
@@ -9352,37 +9323,47 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Centennial Village</t>
+          <t>Brennan Estates</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="E190" t="inlineStr">
-        <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+          <t>Aspen Property Management, MC</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>steve@neighborhoodresources.net</t>
+          <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>302-521-1961</t>
+          <t>410-620-2598</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>https://neighborhoodresources.net</t>
+          <t>https://brennanestatesassociation.org</t>
+        </is>
+      </c>
+      <c r="J190" t="inlineStr">
+        <is>
+          <t>BEAR</t>
+        </is>
+      </c>
+      <c r="K190" t="inlineStr">
+        <is>
+          <t>19701</t>
+        </is>
+      </c>
+      <c r="L190" t="inlineStr">
+        <is>
+          <t>831</t>
         </is>
       </c>
       <c r="M190" t="inlineStr">
@@ -9404,42 +9385,47 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Chaddwyck</t>
+          <t>Centennial Village</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>professionally managed (Premier Community Association Mgmt., MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Premier Community Association Mgmt., MC</t>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>chaddwyckDE@gmail.com</t>
+          <t>steve@neighborhoodresources.net</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>302-449-2230</t>
-        </is>
-      </c>
-      <c r="H191" t="inlineStr">
-        <is>
-          <t>34634 Bay Crossing Boulevard, Suite 4, Lewes, DE 19958</t>
+          <t>302-521-1961</t>
+        </is>
+      </c>
+      <c r="I191" t="inlineStr">
+        <is>
+          <t>https://neighborhoodresources.net</t>
         </is>
       </c>
       <c r="M191" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N191" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -9451,62 +9437,42 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Chandeleur Woods</t>
+          <t>Chaddwyck</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
+          <t>professionally managed (Premier Community Association Mgmt., MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="E192" t="inlineStr">
-        <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+          <t>Premier Community Association Mgmt., MC</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>steve@neighborhoodresources.net</t>
+          <t>chaddwyckDE@gmail.com</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>302-521-1961</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>https://neighborhoodresources.net</t>
-        </is>
-      </c>
-      <c r="J192" t="inlineStr">
-        <is>
-          <t>BEAR</t>
-        </is>
-      </c>
-      <c r="K192" t="inlineStr">
-        <is>
-          <t>19701</t>
-        </is>
-      </c>
-      <c r="L192" t="inlineStr">
-        <is>
-          <t>121</t>
+          <t>302-449-2230</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>34634 Bay Crossing Boulevard, Suite 4, Lewes, DE 19958</t>
         </is>
       </c>
       <c r="M192" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N192" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -9518,32 +9484,37 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Crossings At Christiana</t>
+          <t>Chandeleur Woods</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Brandywine Valley Properties, MC</t>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>info@bvprops.com</t>
+          <t>steve@neighborhoodresources.net</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>302-475-7660</t>
+          <t>302-521-1961</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>http://www.bvprops.com/</t>
+          <t>https://neighborhoodresources.net</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -9558,7 +9529,7 @@
       </c>
       <c r="L193" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>121</t>
         </is>
       </c>
       <c r="M193" t="inlineStr">
@@ -9580,42 +9551,57 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Crossland at the Canal</t>
+          <t>Crossings At Christiana</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>professionally managed (Associa Mid-Atlantic, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Associa Mid-Atlantic, MC</t>
+          <t>Brandywine Valley Properties, MC</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>paula.santangelo@associa.us</t>
+          <t>info@bvprops.com</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>484-754-5706</t>
-        </is>
-      </c>
-      <c r="H194" t="inlineStr">
-        <is>
-          <t>555 Crofton Road, Suite 400, King of Prussia, PA 19406</t>
+          <t>302-475-7660</t>
+        </is>
+      </c>
+      <c r="I194" t="inlineStr">
+        <is>
+          <t>http://www.bvprops.com/</t>
+        </is>
+      </c>
+      <c r="J194" t="inlineStr">
+        <is>
+          <t>BEAR</t>
+        </is>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>19701</t>
+        </is>
+      </c>
+      <c r="L194" t="inlineStr">
+        <is>
+          <t>142</t>
         </is>
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N194" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -9627,37 +9613,32 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Enclave at Odessa</t>
+          <t>Crossland at the Canal</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>professionally managed (Knight Property Services, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Associa Mid-Atlantic, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Knight Property Services, MC</t>
+          <t>Associa Mid-Atlantic, MC</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>mehart@knightpropertysvs.com</t>
+          <t>paula.santangelo@associa.us</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>302-508-2638</t>
+          <t>484-754-5706</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>350 N Hight Street, Smyrna, DE 19977</t>
-        </is>
-      </c>
-      <c r="I195" t="inlineStr">
-        <is>
-          <t>https://bccommunities.org</t>
+          <t>555 Crofton Road, Suite 400, King of Prussia, PA 19406</t>
         </is>
       </c>
       <c r="M195" t="inlineStr">
@@ -9679,57 +9660,47 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Estates At Cedar Lane</t>
+          <t>Enclave at Odessa</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Knight Property Services, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Knight Property Services, MC</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>mehart@knightpropertysvs.com</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
+          <t>302-508-2638</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>350 N Hight Street, Smyrna, DE 19977</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>https://www.aspenpropertymgmt.com</t>
-        </is>
-      </c>
-      <c r="J196" t="inlineStr">
-        <is>
-          <t>MIDDLETOWN</t>
-        </is>
-      </c>
-      <c r="K196" t="inlineStr">
-        <is>
-          <t>19709</t>
-        </is>
-      </c>
-      <c r="L196" t="inlineStr">
-        <is>
-          <t>83</t>
+          <t>https://bccommunities.org</t>
         </is>
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N196" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -9741,7 +9712,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Fairways at Vandegrift</t>
+          <t>Estates At Cedar Lane</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -9764,24 +9735,34 @@
           <t>410-620-2598</t>
         </is>
       </c>
-      <c r="H197" t="inlineStr">
-        <is>
-          <t>14 S Main Street, North East, MD 21901</t>
-        </is>
-      </c>
       <c r="I197" t="inlineStr">
         <is>
           <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
+      <c r="J197" t="inlineStr">
+        <is>
+          <t>MIDDLETOWN</t>
+        </is>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>19709</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr">
+        <is>
+          <t>83</t>
+        </is>
+      </c>
       <c r="M197" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -9793,7 +9774,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Forest Glen II</t>
+          <t>Fairways at Vandegrift</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -9816,34 +9797,24 @@
           <t>410-620-2598</t>
         </is>
       </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>14 S Main Street, North East, MD 21901</t>
+        </is>
+      </c>
       <c r="I198" t="inlineStr">
         <is>
           <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
-      <c r="J198" t="inlineStr">
-        <is>
-          <t>BEAR</t>
-        </is>
-      </c>
-      <c r="K198" t="inlineStr">
-        <is>
-          <t>19701</t>
-        </is>
-      </c>
-      <c r="L198" t="inlineStr">
-        <is>
-          <t>167</t>
-        </is>
-      </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N198" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -9855,52 +9826,57 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Glendale II</t>
+          <t>Forest Glen II</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="E199" t="inlineStr">
-        <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+          <t>Aspen Property Management, MC</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>steve@neighborhoodresources.net</t>
+          <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>302-521-1961</t>
-        </is>
-      </c>
-      <c r="H199" t="inlineStr">
-        <is>
-          <t>P.O. Box 10012, Wilmington, DE 19850</t>
+          <t>410-620-2598</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>https://neighborhoodresources.net</t>
+          <t>https://www.aspenpropertymgmt.com</t>
+        </is>
+      </c>
+      <c r="J199" t="inlineStr">
+        <is>
+          <t>BEAR</t>
+        </is>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>19701</t>
+        </is>
+      </c>
+      <c r="L199" t="inlineStr">
+        <is>
+          <t>167</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -9912,37 +9888,42 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Greenville Overlook</t>
+          <t>Glendale II</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Brandywine Valley Properties, MC</t>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>kathybvp3@gmail.com</t>
+          <t>steve@neighborhoodresources.net</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>302-293-8093</t>
+          <t>302-521-1961</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>P.O. Box 7367, Wilmington, DE 19803</t>
+          <t>P.O. Box 10012, Wilmington, DE 19850</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>https://www.gvol.net</t>
+          <t>https://neighborhoodresources.net</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -9964,37 +9945,37 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Highpointe at St. Georges</t>
+          <t>Greenville Overlook</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>professionally managed (CAMCO Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>CAMCO Management, MC</t>
+          <t>Brandywine Valley Properties, MC</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>info@camcomgmt.com</t>
+          <t>kathybvp3@gmail.com</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>215-942-6621</t>
+          <t>302-293-8093</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>501 W Office Center Drive, Suite 220, Fort Washington, PA 19034</t>
+          <t>P.O. Box 7367, Wilmington, DE 19803</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>https://camcomgmt.com</t>
+          <t>https://www.gvol.net</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -10016,57 +9997,47 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Hockessin Chase</t>
+          <t>Highpointe at St. Georges</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (CAMCO Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Brandywine Valley Properties, MC</t>
+          <t>CAMCO Management, MC</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>info@bvprops.com</t>
+          <t>info@camcomgmt.com</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>302-475-7660</t>
+          <t>215-942-6621</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>501 W Office Center Drive, Suite 220, Fort Washington, PA 19034</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>http://www.bvprops.com</t>
-        </is>
-      </c>
-      <c r="J202" t="inlineStr">
-        <is>
-          <t>HOCKESSIN</t>
-        </is>
-      </c>
-      <c r="K202" t="inlineStr">
-        <is>
-          <t>19707</t>
-        </is>
-      </c>
-      <c r="L202" t="inlineStr">
-        <is>
-          <t>155</t>
+          <t>https://camcomgmt.com</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N202" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -10078,52 +10049,47 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Hyetts Crossing</t>
+          <t>Hockessin Chase</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
+          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="E203" t="inlineStr">
-        <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+          <t>Brandywine Valley Properties, MC</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>steve@neighborhoodresources.net</t>
+          <t>info@bvprops.com</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>302-521-1961</t>
+          <t>302-475-7660</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>https://neighborhoodresources.net</t>
+          <t>http://www.bvprops.com</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
         <is>
-          <t>MIDDLETOWN</t>
+          <t>HOCKESSIN</t>
         </is>
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>19709</t>
+          <t>19707</t>
         </is>
       </c>
       <c r="L203" t="inlineStr">
         <is>
-          <t>323</t>
+          <t>155</t>
         </is>
       </c>
       <c r="M203" t="inlineStr">
@@ -10145,42 +10111,62 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>La Grange</t>
+          <t>Hyetts Crossing</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>professionally managed (c/o CCPMDE, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>c/o CCPMDE, MC</t>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>info@ccpmde.com</t>
-        </is>
-      </c>
-      <c r="H204" t="inlineStr">
-        <is>
-          <t>501 Silverside Road, Suite 38, Wilmington, DE 19809</t>
+          <t>steve@neighborhoodresources.net</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>302-521-1961</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>https://www.lagrangehoa.com</t>
+          <t>https://neighborhoodresources.net</t>
+        </is>
+      </c>
+      <c r="J204" t="inlineStr">
+        <is>
+          <t>MIDDLETOWN</t>
+        </is>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>19709</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr">
+        <is>
+          <t>323</t>
         </is>
       </c>
       <c r="M204" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N204" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -10192,37 +10178,32 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Limestone Hills</t>
+          <t>La Grange</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>professionally managed (Kelly Management Services, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (c/o CCPMDE, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Kelly Management Services, MC</t>
+          <t>c/o CCPMDE, MC</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>lkelly@kellymanagementservices.com</t>
-        </is>
-      </c>
-      <c r="G205" t="inlineStr">
-        <is>
-          <t>302-565-4499</t>
+          <t>info@ccpmde.com</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>312 W State Street, Suite 20, Kennett Square, PA 19348</t>
+          <t>501 Silverside Road, Suite 38, Wilmington, DE 19809</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>https://www.limestonehills.com</t>
+          <t>https://www.lagrangehoa.com</t>
         </is>
       </c>
       <c r="M205" t="inlineStr">
@@ -10244,52 +10225,47 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Little Falls Village</t>
+          <t>Limestone Hills</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>professionally managed (Mastriana Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Kelly Management Services, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Mastriana Property Management, MC</t>
+          <t>Kelly Management Services, MC</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>mastrianapropmgt@aol.com</t>
+          <t>lkelly@kellymanagementservices.com</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>302-234-4860</t>
-        </is>
-      </c>
-      <c r="J206" t="inlineStr">
-        <is>
-          <t>WILMINGTON</t>
-        </is>
-      </c>
-      <c r="K206" t="inlineStr">
-        <is>
-          <t>19808</t>
-        </is>
-      </c>
-      <c r="L206" t="inlineStr">
-        <is>
-          <t>108</t>
+          <t>302-565-4499</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>312 W State Street, Suite 20, Kennett Square, PA 19348</t>
+        </is>
+      </c>
+      <c r="I206" t="inlineStr">
+        <is>
+          <t>https://www.limestonehills.com</t>
         </is>
       </c>
       <c r="M206" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N206" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -10301,52 +10277,42 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Llangollen Green</t>
+          <t>Little Falls Village</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
+          <t>professionally managed (Mastriana Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
-        </is>
-      </c>
-      <c r="E207" t="inlineStr">
-        <is>
-          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+          <t>Mastriana Property Management, MC</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>steve@neighborhoodresources.net</t>
+          <t>mastrianapropmgt@aol.com</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>302-521-1961</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>https://neighborhoodresources.net</t>
+          <t>302-234-4860</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
         <is>
-          <t>NEW CASTLE</t>
+          <t>WILMINGTON</t>
         </is>
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>19720</t>
+          <t>19808</t>
         </is>
       </c>
       <c r="L207" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>108</t>
         </is>
       </c>
       <c r="M207" t="inlineStr">
@@ -10368,7 +10334,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Mallard Pointe</t>
+          <t>Llangollen Green</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -10396,6 +10362,11 @@
           <t>302-521-1961</t>
         </is>
       </c>
+      <c r="I208" t="inlineStr">
+        <is>
+          <t>https://neighborhoodresources.net</t>
+        </is>
+      </c>
       <c r="J208" t="inlineStr">
         <is>
           <t>NEW CASTLE</t>
@@ -10408,7 +10379,7 @@
       </c>
       <c r="L208" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>180</t>
         </is>
       </c>
       <c r="M208" t="inlineStr">
@@ -10430,7 +10401,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Meadow Glen</t>
+          <t>Mallard Pointe</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -10460,17 +10431,17 @@
       </c>
       <c r="J209" t="inlineStr">
         <is>
-          <t>BEAR</t>
+          <t>NEW CASTLE</t>
         </is>
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>19701</t>
+          <t>19720</t>
         </is>
       </c>
       <c r="L209" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>219</t>
         </is>
       </c>
       <c r="M209" t="inlineStr">
@@ -10492,47 +10463,47 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Milltown Village</t>
+          <t>Meadow Glen</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>professionally managed (Investment Property Services, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Neighborhood Resources LLC, Steve Blanchies) [contact is a company name]</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Investment Property Services, MC</t>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Neighborhood Resources LLC, Steve Blanchies</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>cperonti@ipsde.com</t>
+          <t>steve@neighborhoodresources.net</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>302-994-3907</t>
-        </is>
-      </c>
-      <c r="I210" t="inlineStr">
-        <is>
-          <t>https://www.milltownvillage.org</t>
+          <t>302-521-1961</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
         <is>
-          <t>WILMINGTON</t>
+          <t>BEAR</t>
         </is>
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>19808</t>
+          <t>19701</t>
         </is>
       </c>
       <c r="L210" t="inlineStr">
         <is>
-          <t>119</t>
+          <t>63</t>
         </is>
       </c>
       <c r="M210" t="inlineStr">
@@ -10554,47 +10525,47 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Perch Creek</t>
+          <t>Milltown Village</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Investment Property Services, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Investment Property Services, MC</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>cperonti@ipsde.com</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
+          <t>302-994-3907</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>https://www.aspenpropertymgmt.com</t>
+          <t>https://www.milltownvillage.org</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
         <is>
-          <t>NEWARK</t>
+          <t>WILMINGTON</t>
         </is>
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>19702</t>
+          <t>19808</t>
         </is>
       </c>
       <c r="L211" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>119</t>
         </is>
       </c>
       <c r="M211" t="inlineStr">
@@ -10616,47 +10587,57 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Red Lion Chase</t>
+          <t>Perch Creek</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>professionally managed (CAMCO Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>CAMCO Management, MC</t>
+          <t>Aspen Property Management, MC</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>info@camcomgmt.com</t>
+          <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>215-942-6621</t>
-        </is>
-      </c>
-      <c r="H212" t="inlineStr">
-        <is>
-          <t>501 W Office Center Drive, Suite 220, Fort Washington, PA 19034</t>
+          <t>410-620-2598</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>https://camcomgmt.com</t>
+          <t>https://www.aspenpropertymgmt.com</t>
+        </is>
+      </c>
+      <c r="J212" t="inlineStr">
+        <is>
+          <t>NEWARK</t>
+        </is>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>19702</t>
+        </is>
+      </c>
+      <c r="L212" t="inlineStr">
+        <is>
+          <t>200</t>
         </is>
       </c>
       <c r="M212" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N212" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -10668,57 +10649,47 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>River Walk</t>
+          <t>Red Lion Chase</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (CAMCO Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Brandywine Valley Properties, MC</t>
+          <t>CAMCO Management, MC</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>info@bvprops.com</t>
+          <t>info@camcomgmt.com</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>302-475-7660</t>
+          <t>215-942-6621</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>501 W Office Center Drive, Suite 220, Fort Washington, PA 19034</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>http://www.bvprops.com</t>
-        </is>
-      </c>
-      <c r="J213" t="inlineStr">
-        <is>
-          <t>NEWARK</t>
-        </is>
-      </c>
-      <c r="K213" t="inlineStr">
-        <is>
-          <t>19702</t>
-        </is>
-      </c>
-      <c r="L213" t="inlineStr">
-        <is>
-          <t>207</t>
+          <t>https://camcomgmt.com</t>
         </is>
       </c>
       <c r="M213" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N213" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -10730,32 +10701,47 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Rose Hill At Lexington Farms</t>
+          <t>River Walk</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Brandywine Valley Properties, MC</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>info@bvprops.com</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
+          <t>302-475-7660</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>https://www.aspenpropertymgmt.com</t>
+          <t>http://www.bvprops.com</t>
+        </is>
+      </c>
+      <c r="J214" t="inlineStr">
+        <is>
+          <t>NEWARK</t>
+        </is>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>19702</t>
+        </is>
+      </c>
+      <c r="L214" t="inlineStr">
+        <is>
+          <t>207</t>
         </is>
       </c>
       <c r="M214" t="inlineStr">
@@ -10777,47 +10763,42 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Rosetree Hunt</t>
+          <t>Rose Hill At Lexington Farms</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Brandywine Valley Properties, MC</t>
+          <t>Aspen Property Management, MC</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>info@bvprops.com</t>
+          <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>302-475-7660</t>
-        </is>
-      </c>
-      <c r="H215" t="inlineStr">
-        <is>
-          <t>P.O. Box 7368, Wilmington, DE 19803</t>
+          <t>410-620-2598</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>http://www.bvprops.com</t>
+          <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="M215" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N215" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -10829,57 +10810,47 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Shannon Cove</t>
+          <t>Rosetree Hunt</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Brandywine Valley Properties, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Brandywine Valley Properties, MC</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>info@bvprops.com</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
+          <t>302-475-7660</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>P.O. Box 7368, Wilmington, DE 19803</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>https://www.aspenpropertymgmt.com</t>
-        </is>
-      </c>
-      <c r="J216" t="inlineStr">
-        <is>
-          <t>MIDDLETOWN</t>
-        </is>
-      </c>
-      <c r="K216" t="inlineStr">
-        <is>
-          <t>19709</t>
-        </is>
-      </c>
-      <c r="L216" t="inlineStr">
-        <is>
-          <t>422</t>
+          <t>http://www.bvprops.com</t>
         </is>
       </c>
       <c r="M216" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N216" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -10891,32 +10862,47 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Stone Mill</t>
+          <t>Shannon Cove</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>professionally managed (Associa Mid-Atlantic, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Associa Mid-Atlantic, MC</t>
+          <t>Aspen Property Management, MC</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>info@aspenpropertymgmt.com</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>410-620-2598</t>
+        </is>
+      </c>
+      <c r="I217" t="inlineStr">
+        <is>
+          <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
         <is>
-          <t>BEAR</t>
+          <t>MIDDLETOWN</t>
         </is>
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>19701</t>
+          <t>19709</t>
         </is>
       </c>
       <c r="L217" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>422</t>
         </is>
       </c>
       <c r="M217" t="inlineStr">
@@ -10938,47 +10924,42 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Stonewold</t>
+          <t>Stone Mill</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>professionally managed (A2Z Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Associa Mid-Atlantic, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>A2Z Property Management, MC</t>
-        </is>
-      </c>
-      <c r="F218" t="inlineStr">
-        <is>
-          <t>stonewold@a2zpmc.com</t>
-        </is>
-      </c>
-      <c r="G218" t="inlineStr">
-        <is>
-          <t>302-239-6000</t>
-        </is>
-      </c>
-      <c r="H218" t="inlineStr">
-        <is>
-          <t>P.O. Box 1376, Hockessin, DE 19707</t>
-        </is>
-      </c>
-      <c r="I218" t="inlineStr">
-        <is>
-          <t>https://a2zpmc.com</t>
+          <t>Associa Mid-Atlantic, MC</t>
+        </is>
+      </c>
+      <c r="J218" t="inlineStr">
+        <is>
+          <t>BEAR</t>
+        </is>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>19701</t>
+        </is>
+      </c>
+      <c r="L218" t="inlineStr">
+        <is>
+          <t>203</t>
         </is>
       </c>
       <c r="M218" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N218" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -10990,27 +10971,37 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>The Ridge</t>
+          <t>Stonewold</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>professionally managed (Mastriana Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (A2Z Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Mastriana Property Management, MC</t>
+          <t>A2Z Property Management, MC</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>stonewold@a2zpmc.com</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>302-234-4860</t>
+          <t>302-239-6000</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>5500 Skyline Drive, Suite 6, Wilmington, DE 19801</t>
+          <t>P.O. Box 1376, Hockessin, DE 19707</t>
+        </is>
+      </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>https://a2zpmc.com</t>
         </is>
       </c>
       <c r="M219" t="inlineStr">
@@ -11032,57 +11023,37 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Village Of Bayberry North</t>
+          <t>The Ridge</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>professionally managed (Premier Community Association Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Mastriana Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Premier Community Association Management, MC</t>
-        </is>
-      </c>
-      <c r="F220" t="inlineStr">
-        <is>
-          <t>jgoodyear@pcam.net</t>
+          <t>Mastriana Property Management, MC</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>302-449-2230</t>
-        </is>
-      </c>
-      <c r="I220" t="inlineStr">
-        <is>
-          <t>https://premierpropertyandpool.com</t>
-        </is>
-      </c>
-      <c r="J220" t="inlineStr">
-        <is>
-          <t>MIDDLETOWN</t>
-        </is>
-      </c>
-      <c r="K220" t="inlineStr">
-        <is>
-          <t>19709</t>
-        </is>
-      </c>
-      <c r="L220" t="inlineStr">
-        <is>
-          <t>1000</t>
+          <t>302-234-4860</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>5500 Skyline Drive, Suite 6, Wilmington, DE 19801</t>
         </is>
       </c>
       <c r="M220" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N220" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -11094,7 +11065,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Village Of Bayberry South</t>
+          <t>Village Of Bayberry North</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -11156,47 +11127,57 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Village of Rocky Run Condos</t>
+          <t>Village Of Bayberry South</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>professionally managed (Penco Management Inc., MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Premier Community Association Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Penco Management Inc., MC</t>
+          <t>Premier Community Association Management, MC</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>rwhite@pencomanagement.co</t>
+          <t>jgoodyear@pcam.net</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
         <is>
-          <t>610-358-5580</t>
-        </is>
-      </c>
-      <c r="H222" t="inlineStr">
-        <is>
-          <t>5 Christy Drive, Chadds Ford, PA 19317</t>
+          <t>302-449-2230</t>
         </is>
       </c>
       <c r="I222" t="inlineStr">
         <is>
-          <t>https://pencomanagement.com</t>
+          <t>https://premierpropertyandpool.com</t>
+        </is>
+      </c>
+      <c r="J222" t="inlineStr">
+        <is>
+          <t>MIDDLETOWN</t>
+        </is>
+      </c>
+      <c r="K222" t="inlineStr">
+        <is>
+          <t>19709</t>
+        </is>
+      </c>
+      <c r="L222" t="inlineStr">
+        <is>
+          <t>1000</t>
         </is>
       </c>
       <c r="M222" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>cold</t>
         </is>
       </c>
       <c r="N222" t="inlineStr">
         <is>
-          <t>nccde_association_directory</t>
+          <t>nccde_parcel_subdiv</t>
         </is>
       </c>
     </row>
@@ -11208,57 +11189,47 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Woodland Village</t>
+          <t>Village of Rocky Run Condos</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+          <t>professionally managed (Penco Management Inc., MC) [directory 'MC' marker]</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Aspen Property Management, MC</t>
+          <t>Penco Management Inc., MC</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>info@aspenpropertymgmt.com</t>
+          <t>rwhite@pencomanagement.co</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
         <is>
-          <t>410-620-2598</t>
+          <t>610-358-5580</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>5 Christy Drive, Chadds Ford, PA 19317</t>
         </is>
       </c>
       <c r="I223" t="inlineStr">
         <is>
-          <t>https://www.aspenpropertymgmt.com</t>
-        </is>
-      </c>
-      <c r="J223" t="inlineStr">
-        <is>
-          <t>NEWARK</t>
-        </is>
-      </c>
-      <c r="K223" t="inlineStr">
-        <is>
-          <t>19702</t>
-        </is>
-      </c>
-      <c r="L223" t="inlineStr">
-        <is>
-          <t>147</t>
+          <t>https://pencomanagement.com</t>
         </is>
       </c>
       <c r="M223" t="inlineStr">
         <is>
-          <t>cold</t>
+          <t>new</t>
         </is>
       </c>
       <c r="N223" t="inlineStr">
         <is>
-          <t>nccde_parcel_subdiv</t>
+          <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
@@ -11270,52 +11241,114 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
+          <t>Woodland Village</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>Aspen Property Management, MC</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>info@aspenpropertymgmt.com</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>410-620-2598</t>
+        </is>
+      </c>
+      <c r="I224" t="inlineStr">
+        <is>
+          <t>https://www.aspenpropertymgmt.com</t>
+        </is>
+      </c>
+      <c r="J224" t="inlineStr">
+        <is>
+          <t>NEWARK</t>
+        </is>
+      </c>
+      <c r="K224" t="inlineStr">
+        <is>
+          <t>19702</t>
+        </is>
+      </c>
+      <c r="L224" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>nccde_parcel_subdiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="5" t="inlineStr">
+        <is>
+          <t>3 - professionally managed</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
           <t>Wynthrope</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr">
+      <c r="C225" t="inlineStr">
         <is>
           <t>professionally managed (Aspen Property Management, MC) [directory 'MC' marker]</t>
         </is>
       </c>
-      <c r="D224" t="inlineStr">
+      <c r="D225" t="inlineStr">
         <is>
           <t>Aspen Property Management, MC</t>
         </is>
       </c>
-      <c r="F224" t="inlineStr">
+      <c r="F225" t="inlineStr">
         <is>
           <t>info@aspenpropertymgmt.com</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr">
+      <c r="G225" t="inlineStr">
         <is>
           <t>410-620-2598</t>
         </is>
       </c>
-      <c r="H224" t="inlineStr">
+      <c r="H225" t="inlineStr">
         <is>
           <t>14 S Main Street, North East, MD 21901</t>
         </is>
       </c>
-      <c r="I224" t="inlineStr">
+      <c r="I225" t="inlineStr">
         <is>
           <t>https://www.aspenpropertymgmt.com</t>
         </is>
       </c>
-      <c r="M224" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="N224" t="inlineStr">
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
         <is>
           <t>nccde_association_directory</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N224"/>
+  <autoFilter ref="A1:N225"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>